<commit_message>
solve: na plan_controle_folha_pag_analitico_app ajustado a liberação dos projetos por empresa
</commit_message>
<xml_diff>
--- a/df_group_desc_tipo_placa.xlsx
+++ b/df_group_desc_tipo_placa.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>handle_nivel_superior</t>
+  </si>
   <si>
     <t>desc_tipo_veic</t>
   </si>
@@ -380,25 +383,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
+      <c r="B2">
+        <v>1267</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2">
         <v>-267697.25</v>
       </c>
     </row>

</xml_diff>